<commit_message>
Add phone number validation for manuaal bank transfer
</commit_message>
<xml_diff>
--- a/apps/rahat-ui/public/files/verify-payout-sample.xlsx
+++ b/apps/rahat-ui/public/files/verify-payout-sample.xlsx
@@ -20,32 +20,35 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t xml:space="preserve">Amount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bank Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bank Account Number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bank Account Holder Name </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approval Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transaction Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date</t>
-  </si>
-</sst>
+<ns0:sst xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+  <ns0:si>
+    <ns0:t xml:space="preserve">Amount</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Remark</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Bank Name</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Bank Account Number</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Bank Account Holder Name </ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Approval Date</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Transaction Status</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Date</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Phone Number</ns0:t>
+  </ns0:si>
+</ns0:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -254,59 +257,62 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultColWidth="12.640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="33.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="41.26"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="D1">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>LEN(TRIM(D1))&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetPr filterMode="false">
+    <ns0:pageSetUpPr fitToPage="false"/>
+  </ns0:sheetPr>
+  <ns0:dimension ref="A1:H1"/>
+  <ns0:sheetFormatPr defaultColWidth="12.640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <ns0:cols>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.74"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.86"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="33.2"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40.85"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26.53"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="41.26"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A1" s="1" t="s">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="B1" s="2" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="C1" s="3" t="s">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="D1" s="4" t="s">
+        <ns0:v>3</ns0:v>
+      </ns0:c>
+      <ns0:c r="E1" s="1" t="s">
+        <ns0:v>4</ns0:v>
+      </ns0:c>
+      <ns0:c r="F1" s="5" t="s">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="G1" s="5" t="s">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+      <ns0:c r="H1" s="5" t="s">
+        <ns0:v>7</ns0:v>
+      </ns0:c>
+      <ns0:c r="I1" t="s">
+        <ns0:v>8</ns0:v>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:conditionalFormatting sqref="D1">
+    <ns0:cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <ns0:formula>LEN(TRIM(D1))&gt;0</ns0:formula>
+    </ns0:cfRule>
+  </ns0:conditionalFormatting>
+  <ns0:printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <ns0:pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <ns0:pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <ns0:headerFooter differentFirst="false" differentOddEven="false">
+    <ns0:oddHeader/>
+    <ns0:oddFooter/>
+  </ns0:headerFooter>
+</ns0:worksheet>
 </file>
</xml_diff>